<commit_message>
12.20.25 updates with data viz dashboards
</commit_message>
<xml_diff>
--- a/data/cv_entries.xlsx
+++ b/data/cv_entries.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimwright/Desktop/Resume/wright_cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D23AADE-F79F-2C4A-B901-BF42EB2D0FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4BD48A5-A042-7F4F-A9C7-FBACC373762D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16320" xr2:uid="{C4D43CE4-6AA2-144D-A346-CE8B2E756935}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16160" xr2:uid="{C4D43CE4-6AA2-144D-A346-CE8B2E756935}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="148">
   <si>
     <t>type</t>
   </si>
@@ -418,6 +418,66 @@
   </si>
   <si>
     <t>https://jim-asr.shinyapps.io/KernCountyImmunizationCoalition_SurveyResults/</t>
+  </si>
+  <si>
+    <t>data_viz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First 5 Lake Dolly Parton Imagination Library Geographic Analysis </t>
+  </si>
+  <si>
+    <t>Developed geographic visualization to support First 5 Lake's analysis of countywide reach of Dolly Parton Imagination Library program.</t>
+  </si>
+  <si>
+    <t>https://jim-asr.shinyapps.io/F5Lake_DPIL_Map/</t>
+  </si>
+  <si>
+    <t>First 5 Siskiyou Dolly Parton Imagination Library Survey</t>
+  </si>
+  <si>
+    <t>https://jim-asr.shinyapps.io/F5Siskiyou_DPIL_FY2025-26/</t>
+  </si>
+  <si>
+    <t>First 5 Yuba Strategic Planning Community Survey</t>
+  </si>
+  <si>
+    <t>https://jim-asr.shinyapps.io/yuba_priorities_map/</t>
+  </si>
+  <si>
+    <t>First 5 Kern ASQ Results, FY 2024-25</t>
+  </si>
+  <si>
+    <t>Developed dashboard for First 5 Siskiyou to analyze geographic trends in results to Dolly Parton Imagination Library participant survey.</t>
+  </si>
+  <si>
+    <t>Developed dashboard to display countywide results from Ages and Stages Questionnaire administered during 2024-25 fiscal year.</t>
+  </si>
+  <si>
+    <t>https://jim-asr.shinyapps.io/F5Kern_ASQResults_FY24-25_dashboard/</t>
+  </si>
+  <si>
+    <t>First 5 Kern Immunization Coalition Parent Survey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Developed data dashboard to display results from parent survey on childcare needs and preferences </t>
+  </si>
+  <si>
+    <t>First 5 Kern Disapirities Map</t>
+  </si>
+  <si>
+    <t>Santa Cruz County Office of Education Parent Survey on Childcare Preferences and Needs</t>
+  </si>
+  <si>
+    <t>Co-developed geographic visualization of Kern County community indicators to communicate disparities between zip codes</t>
+  </si>
+  <si>
+    <t>https://www.first5kern.org/investments/#Disparities</t>
+  </si>
+  <si>
+    <t>Developed dashboard to display geographic tends from community survey priority ratings to inform 2026-2031 strategic planning.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Developed data dashboard to display results from parent survey on vaccine beliefs and decision-making </t>
   </si>
 </sst>
 </file>
@@ -462,13 +522,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -785,7 +848,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8559F42B-99AA-F44B-B1DC-6C413C767572}">
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="16384" width="20.83203125" style="1"/>
@@ -1518,7 +1581,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:9" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>86</v>
       </c>
@@ -1536,9 +1599,6 @@
       </c>
       <c r="F42" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="238" x14ac:dyDescent="0.2">
@@ -1560,9 +1620,6 @@
       <c r="F43" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="G43" s="1" t="s">
-        <v>126</v>
-      </c>
     </row>
     <row r="44" spans="1:9" ht="187" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
@@ -1784,6 +1841,167 @@
       </c>
       <c r="I52" s="1" t="s">
         <v>96</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+      <c r="A53" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B53" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C53" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+      <c r="A54" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B54" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C54" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+      <c r="A55" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B55" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C55" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+      <c r="A56" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B56" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C56" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+      <c r="A57" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B57" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C57" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="85" x14ac:dyDescent="0.2">
+      <c r="A58" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B58" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C58" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="136" x14ac:dyDescent="0.2">
+      <c r="A59" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B59" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C59" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
12.21.25 - additional publication and reports added
</commit_message>
<xml_diff>
--- a/data/cv_entries.xlsx
+++ b/data/cv_entries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimwright/Desktop/Resume/wright_cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4BD48A5-A042-7F4F-A9C7-FBACC373762D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC4CBB1E-FA60-AE4B-A110-75030C758521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16160" xr2:uid="{C4D43CE4-6AA2-144D-A346-CE8B2E756935}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="148">
   <si>
     <t>type</t>
   </si>
@@ -1581,7 +1581,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="409.5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>86</v>
       </c>
@@ -1599,6 +1599,9 @@
       </c>
       <c r="F42" s="1" t="s">
         <v>124</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="238" x14ac:dyDescent="0.2">
@@ -1619,6 +1622,9 @@
       </c>
       <c r="F43" s="1" t="s">
         <v>125</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="187" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
ASR Senior Manager promotion
</commit_message>
<xml_diff>
--- a/data/cv_entries.xlsx
+++ b/data/cv_entries.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimwright/Desktop/Resume/wright_cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC4CBB1E-FA60-AE4B-A110-75030C758521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAFEB33C-1AE5-4F4A-96AB-F552DFC1D146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16160" xr2:uid="{C4D43CE4-6AA2-144D-A346-CE8B2E756935}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="150">
   <si>
     <t>type</t>
   </si>
@@ -478,6 +478,13 @@
   </si>
   <si>
     <t xml:space="preserve">Developed data dashboard to display results from parent survey on vaccine beliefs and decision-making </t>
+  </si>
+  <si>
+    <t>Senior Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lead the execution and strategic oversight of complex, mixed-methods research and evaluation initiatives across public health, early childhood, and community-based service systems. Fully manage project scopes of work including timelines, analytic workflows, budgets, and interdisciplinary teams, ensuring alignment between research design, stakeholder needs, and implementation outcomes. Direct the development of survey instruments, qualitative protocols, and data processing pipelines; oversee data cleaning, integration, and analysis across multi-source datasets (e.g., administrative records, survey responses, and public-use data such as Census or state-level reporting systems). Collaborate with program partners and technical staff to translate analytic findings into actionable recommendations through reports, dashboards, and stakeholder-facing presentations. Supervise project staff in reproducible research practices, including R-based data pipelines, version-controlled workflows, and structured documentation to support transparency, replication, and long-term maintainability of analytic outputs. Maintain partner relationships across county agencies and nonprofit service providers, proactively identifying analytic risks and implementation barriers while supporting adaptive decision-making throughout the project lifecycle.
+</t>
   </si>
 </sst>
 </file>
@@ -848,7 +855,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8559F42B-99AA-F44B-B1DC-6C413C767572}">
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="16384" width="20.83203125" style="1"/>
@@ -945,84 +952,84 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="409.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" ht="409" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>120</v>
+        <v>148</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="170" x14ac:dyDescent="0.2">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C7" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="187" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="170" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B8" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C8" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>77</v>
+        <v>115</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>73</v>
+        <v>116</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="170" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="187" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B9" s="1">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C9" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>16</v>
+        <v>77</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>17</v>
+        <v>73</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>67</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="170" x14ac:dyDescent="0.2">
@@ -1030,47 +1037,47 @@
         <v>14</v>
       </c>
       <c r="B10" s="1">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C10" s="1">
         <v>2023</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="170" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="1">
+        <v>2022</v>
+      </c>
+      <c r="C11" s="1">
+        <v>2023</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>118</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="102" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="1">
-        <v>2016</v>
-      </c>
-      <c r="C11" s="1">
-        <v>2017</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B12" s="1">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="C12" s="1">
         <v>2017</v>
@@ -1079,53 +1086,53 @@
         <v>20</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B13" s="1">
         <v>2015</v>
       </c>
       <c r="C13" s="1">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="68" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B14" s="1">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="C14" s="1">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="136" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -1133,150 +1140,153 @@
         <v>2014</v>
       </c>
       <c r="C15" s="1">
+        <v>2015</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="136" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="1">
         <v>2014</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="C16" s="1">
+        <v>2014</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="204" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B16" s="1">
-        <v>2020</v>
-      </c>
-      <c r="C16" s="1">
-        <v>2021</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="221" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" ht="204" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B17" s="1">
-        <v>2018</v>
+        <v>2020</v>
       </c>
       <c r="C17" s="1">
         <v>2021</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="187" x14ac:dyDescent="0.2">
+        <v>33</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="221" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B18" s="1">
+        <v>2018</v>
+      </c>
+      <c r="C18" s="1">
+        <v>2021</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="187" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="1">
         <v>2013</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C19" s="1">
         <v>2014</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D19" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E19" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B19" s="1">
-        <v>2022</v>
-      </c>
-      <c r="C19" s="1">
-        <v>2022</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>70</v>
       </c>
       <c r="B20" s="1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C20" s="1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="B21" s="1">
-        <v>2017</v>
+        <v>2021</v>
       </c>
       <c r="C21" s="1">
         <v>2021</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>30</v>
+      <c r="D21" s="2" t="s">
+        <v>60</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="G21" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B22" s="1">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="C22" s="1">
         <v>2021</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>17</v>
@@ -1287,39 +1297,36 @@
         <v>28</v>
       </c>
       <c r="B23" s="1">
+        <v>2018</v>
+      </c>
+      <c r="C23" s="1">
+        <v>2021</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" s="1">
         <v>2014</v>
       </c>
-      <c r="C23" s="1">
+      <c r="C24" s="1">
         <v>2014</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D24" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="E24" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="221" x14ac:dyDescent="0.2">
-      <c r="A24" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B24" s="1">
-        <v>2018</v>
-      </c>
-      <c r="C24" s="1">
-        <v>2021</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="136" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" ht="221" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>32</v>
       </c>
@@ -1327,50 +1334,53 @@
         <v>2018</v>
       </c>
       <c r="C25" s="1">
+        <v>2021</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="136" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="1">
+        <v>2018</v>
+      </c>
+      <c r="C26" s="1">
         <v>2019</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D26" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="E26" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="F26" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="119" x14ac:dyDescent="0.2">
-      <c r="A26" s="1" t="s">
+    <row r="27" spans="1:7" ht="119" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B27" s="1">
         <v>2015</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C27" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D27" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A27" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B27" s="1">
-        <v>2022</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>42</v>
       </c>
@@ -1381,27 +1391,27 @@
         <v>15</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B29" s="1">
-        <v>2017</v>
+        <v>2022</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>43</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -1409,7 +1419,7 @@
         <v>42</v>
       </c>
       <c r="B30" s="1">
-        <v>2015</v>
+        <v>2017</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>15</v>
@@ -1418,10 +1428,10 @@
         <v>66</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>42</v>
       </c>
@@ -1432,24 +1442,27 @@
         <v>15</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B32" s="1">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="51" x14ac:dyDescent="0.2">
@@ -1457,33 +1470,33 @@
         <v>47</v>
       </c>
       <c r="B33" s="1">
-        <v>2017</v>
+        <v>2014</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D33" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B34" s="1">
+        <v>2017</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="E34" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="136" x14ac:dyDescent="0.2">
-      <c r="A34" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C34" s="1">
-        <v>2019</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="272" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" ht="136" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>50</v>
       </c>
@@ -1491,24 +1504,24 @@
         <v>2019</v>
       </c>
       <c r="D35" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="272" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C36" s="1">
+        <v>2019</v>
+      </c>
+      <c r="D36" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="F36" s="1" t="s">
         <v>54</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A36" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B36" s="1">
-        <v>2010</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1516,13 +1529,13 @@
         <v>79</v>
       </c>
       <c r="B37" s="1">
-        <v>2017</v>
+        <v>2010</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1530,13 +1543,13 @@
         <v>79</v>
       </c>
       <c r="B38" s="1">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1544,13 +1557,13 @@
         <v>79</v>
       </c>
       <c r="B39" s="1">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1558,13 +1571,13 @@
         <v>79</v>
       </c>
       <c r="B40" s="1">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="17" x14ac:dyDescent="0.2">
@@ -1572,39 +1585,30 @@
         <v>79</v>
       </c>
       <c r="B41" s="1">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="B42" s="1">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="I42" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="238" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>86</v>
       </c>
@@ -1615,42 +1619,42 @@
         <v>15</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I43" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="187" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:9" ht="238" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>86</v>
       </c>
       <c r="B44" s="1">
-        <v>2023</v>
-      </c>
-      <c r="C44" s="1">
         <v>2024</v>
       </c>
+      <c r="C44" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="D44" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>73</v>
+        <v>116</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" ht="238" x14ac:dyDescent="0.2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="187" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>86</v>
       </c>
@@ -1661,19 +1665,19 @@
         <v>2024</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>87</v>
+        <v>113</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>88</v>
+        <v>114</v>
       </c>
       <c r="I45" s="1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="255" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:9" ht="238" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>86</v>
       </c>
@@ -1684,48 +1688,45 @@
         <v>2024</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" ht="238" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="255" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>86</v>
       </c>
       <c r="B47" s="1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C47" s="1">
         <v>2024</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" ht="153" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="238" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>86</v>
       </c>
@@ -1736,22 +1737,22 @@
         <v>2024</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" ht="289" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="153" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>86</v>
       </c>
@@ -1762,50 +1763,50 @@
         <v>2024</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" ht="187" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="289" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="B50" s="1">
         <v>2022</v>
       </c>
       <c r="C50" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" ht="323" x14ac:dyDescent="0.2">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="187" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="B51" s="1">
         <v>2022</v>
@@ -1814,19 +1815,22 @@
         <v>2023</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>98</v>
+        <v>105</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>112</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" ht="323" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>86</v>
       </c>
@@ -1837,39 +1841,39 @@
         <v>2023</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F52" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="I52" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+      <c r="A53" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B53" s="1">
+        <v>2022</v>
+      </c>
+      <c r="C53" s="1">
+        <v>2023</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="I52" s="1" t="s">
+      <c r="I53" s="1" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" ht="119" x14ac:dyDescent="0.2">
-      <c r="A53" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B53" s="1">
-        <v>2025</v>
-      </c>
-      <c r="C53" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="54" spans="1:9" ht="119" x14ac:dyDescent="0.2">
@@ -1883,19 +1887,19 @@
         <v>2025</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>128</v>
       </c>
@@ -1906,16 +1910,16 @@
         <v>2025</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="56" spans="1:9" ht="102" x14ac:dyDescent="0.2">
@@ -1929,16 +1933,16 @@
         <v>2025</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="102" x14ac:dyDescent="0.2">
@@ -1952,42 +1956,42 @@
         <v>2025</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" ht="85" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>128</v>
       </c>
       <c r="B58" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C58" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="G58" s="3" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" ht="136" x14ac:dyDescent="0.2">
+        <v>147</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="85" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>128</v>
       </c>
@@ -1998,25 +2002,48 @@
         <v>2024</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F59" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="G59" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="136" x14ac:dyDescent="0.2">
+      <c r="A60" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B60" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C60" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="G59" s="1" t="s">
+      <c r="G60" s="1" t="s">
         <v>145</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F16" r:id="rId1" xr:uid="{9FC96BBB-E6A2-B445-A8BC-D5C33750B0BD}"/>
-    <hyperlink ref="G20" r:id="rId2" xr:uid="{67F88AC2-2CFE-FA4A-92CE-3F4ED8A9D293}"/>
-    <hyperlink ref="D20" r:id="rId3" xr:uid="{67C34580-503B-904D-B129-0E6417699D1E}"/>
-    <hyperlink ref="G19" r:id="rId4" xr:uid="{A592B2D5-64F7-D24F-B190-D84D29F1718E}"/>
-    <hyperlink ref="D19" r:id="rId5" xr:uid="{D42F41A6-5D73-B344-9F8A-BD6292306C55}"/>
+    <hyperlink ref="G21" r:id="rId1" xr:uid="{67F88AC2-2CFE-FA4A-92CE-3F4ED8A9D293}"/>
+    <hyperlink ref="D21" r:id="rId2" xr:uid="{67C34580-503B-904D-B129-0E6417699D1E}"/>
+    <hyperlink ref="G20" r:id="rId3" xr:uid="{A592B2D5-64F7-D24F-B190-D84D29F1718E}"/>
+    <hyperlink ref="D20" r:id="rId4" xr:uid="{D42F41A6-5D73-B344-9F8A-BD6292306C55}"/>
+    <hyperlink ref="F17" r:id="rId5" xr:uid="{9FC96BBB-E6A2-B445-A8BC-D5C33750B0BD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
4.29 addition of SRA dashboard
</commit_message>
<xml_diff>
--- a/data/cv_entries.xlsx
+++ b/data/cv_entries.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimwright/Desktop/Resume/wright_cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAFEB33C-1AE5-4F4A-96AB-F552DFC1D146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D608FC9-0607-5741-A2FF-09D72508B3F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16160" xr2:uid="{C4D43CE4-6AA2-144D-A346-CE8B2E756935}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="153">
   <si>
     <t>type</t>
   </si>
@@ -405,13 +405,7 @@
     <t>Lake, Kern, Siskiyou, Sutter, Yuba, and Ventura Counties, CA</t>
   </si>
   <si>
-    <t>Butte, Plumas, and Santa Cruz County Offices of Education, CA</t>
-  </si>
-  <si>
     <t>Lead Project Manager for ASR's consulting work with six California First 5 County Commissions. Support Commission efforts related to annual program evaluation, including data collection, management, analysis, and reporting. Facilitate strategic planning initiatives, including the design and distribution of surveys via Qualtrics and the collection of qualitative data through focus groups and key informant interviews. Spearhead special projects, including the design, implementation, and analysis of key surveys such as the First 5 Kern Developmental Screening Gap Assessment and the Parent/Guardian Survey and Vaccination and Immunization for the Kery County Immunization Coalition.</t>
-  </si>
-  <si>
-    <t>Serve as Lead Project Manager for ASR's consulting work with three California County Offices of Education. Oversee the design and execution of Needs Assessments and parent surveys focused on perceptions, barriers, and priorities related to child care availability, priorities, and barriers to access.</t>
   </si>
   <si>
     <t>https://jim-asr.shinyapps.io/SantaCruz_UPK_Survey/</t>
@@ -485,6 +479,21 @@
   <si>
     <t xml:space="preserve">Lead the execution and strategic oversight of complex, mixed-methods research and evaluation initiatives across public health, early childhood, and community-based service systems. Fully manage project scopes of work including timelines, analytic workflows, budgets, and interdisciplinary teams, ensuring alignment between research design, stakeholder needs, and implementation outcomes. Direct the development of survey instruments, qualitative protocols, and data processing pipelines; oversee data cleaning, integration, and analysis across multi-source datasets (e.g., administrative records, survey responses, and public-use data such as Census or state-level reporting systems). Collaborate with program partners and technical staff to translate analytic findings into actionable recommendations through reports, dashboards, and stakeholder-facing presentations. Supervise project staff in reproducible research practices, including R-based data pipelines, version-controlled workflows, and structured documentation to support transparency, replication, and long-term maintainability of analytic outputs. Maintain partner relationships across county agencies and nonprofit service providers, proactively identifying analytic risks and implementation barriers while supporting adaptive decision-making throughout the project lifecycle.
 </t>
+  </si>
+  <si>
+    <t>Butte, Plumas, Santa Cruz, and Tehama County Offices of Education, CA</t>
+  </si>
+  <si>
+    <t>Serve as Lead Project Manager for ASR's consulting work with four California County Offices of Education. Oversee the design and execution of Needs Assessments and parent surveys focused on perceptions, barriers, and priorities related to child care availability, priorities, and barriers to access.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First 5 Siskiyou School Readiness and Third Grade Reading Proficiency </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Developed longitudinal, geographic summary of First 5 Siskiyou's Kindergarten Readiness Assessment results to compare to trends in countywide Third Grade reading proficiency. </t>
+  </si>
+  <si>
+    <t>https://jim-asr.shinyapps.io/F5Siskiyou_ELA_Readiness_Dashboard/</t>
   </si>
 </sst>
 </file>
@@ -559,9 +568,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -599,7 +608,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -705,7 +714,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -847,7 +856,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -855,7 +864,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8559F42B-99AA-F44B-B1DC-6C413C767572}">
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="16384" width="20.83203125" style="1"/>
@@ -963,13 +972,13 @@
         <v>15</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="409.5" x14ac:dyDescent="0.2">
@@ -1625,7 +1634,7 @@
         <v>116</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I43" s="1" t="s">
         <v>120</v>
@@ -1642,13 +1651,13 @@
         <v>15</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
       <c r="I44" s="1" t="s">
         <v>120</v>
@@ -1876,32 +1885,32 @@
         <v>96</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:9" ht="136" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B54" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C54" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B55" s="1">
         <v>2025</v>
@@ -1910,21 +1919,21 @@
         <v>2025</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B56" s="1">
         <v>2025</v>
@@ -1933,21 +1942,21 @@
         <v>2025</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B57" s="1">
         <v>2025</v>
@@ -1956,21 +1965,21 @@
         <v>2025</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
     </row>
     <row r="58" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B58" s="1">
         <v>2025</v>
@@ -1979,44 +1988,44 @@
         <v>2025</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" ht="85" x14ac:dyDescent="0.2">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B59" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C59" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="G59" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="85" x14ac:dyDescent="0.2">
+      <c r="A60" s="1" t="s">
         <v>126</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" ht="136" x14ac:dyDescent="0.2">
-      <c r="A60" s="1" t="s">
-        <v>128</v>
       </c>
       <c r="B60" s="1">
         <v>2024</v>
@@ -2025,16 +2034,39 @@
         <v>2024</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>116</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>145</v>
+        <v>139</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" ht="136" x14ac:dyDescent="0.2">
+      <c r="A61" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B61" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C61" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
7.12 removal of MZR shiny app links
</commit_message>
<xml_diff>
--- a/data/cv_entries.xlsx
+++ b/data/cv_entries.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimwright/Desktop/Resume/wright_cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D608FC9-0607-5741-A2FF-09D72508B3F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B58EA9AD-27DA-E848-B503-047BC173AFD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16160" xr2:uid="{C4D43CE4-6AA2-144D-A346-CE8B2E756935}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="148">
   <si>
     <t>type</t>
   </si>
@@ -354,25 +354,10 @@
     <t>Responsible for data collection and analysis through survey administration and focus group facilitation. Also supported the identification of positive outlier schools through analysis of school proficiency ratings.</t>
   </si>
   <si>
-    <t>https://marzanoresearch.shinyapps.io/all_districts/</t>
-  </si>
-  <si>
-    <t>https://marzanoresearch.shinyapps.io/ks_version4/</t>
-  </si>
-  <si>
     <t>Wyoming Believing in Literacy Together (WY BILT)</t>
   </si>
   <si>
     <t>Responsible for providing professional development sessions as a methodologist to assist participating teachers design and implement research studies within their classrooms. As a data analyst, responsible for the evaluation and communication of exit survey data to inform and influence improvements to the professional learning series.</t>
-  </si>
-  <si>
-    <t>https://marzanoresearch.shinyapps.io/cohort1_exit_survey/</t>
-  </si>
-  <si>
-    <t>https://marzanoresearch.shinyapps.io/wy_bilt_v2/</t>
-  </si>
-  <si>
-    <t>https://marzanoresearch.shinyapps.io/wy_act_school_movement/</t>
   </si>
   <si>
     <t>Rapid City, SD Area Schools Special Education Program Review</t>
@@ -568,9 +553,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -608,7 +593,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -714,7 +699,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -856,7 +841,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -972,13 +957,13 @@
         <v>15</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="409.5" x14ac:dyDescent="0.2">
@@ -992,13 +977,13 @@
         <v>2026</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="170" x14ac:dyDescent="0.2">
@@ -1012,13 +997,13 @@
         <v>2025</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="187" x14ac:dyDescent="0.2">
@@ -1038,7 +1023,7 @@
         <v>73</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="170" x14ac:dyDescent="0.2">
@@ -1078,7 +1063,7 @@
         <v>73</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="102" x14ac:dyDescent="0.2">
@@ -1617,7 +1602,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:9" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>86</v>
       </c>
@@ -1628,16 +1613,16 @@
         <v>15</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="238" x14ac:dyDescent="0.2">
@@ -1651,16 +1636,16 @@
         <v>15</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="187" x14ac:dyDescent="0.2">
@@ -1674,13 +1659,13 @@
         <v>2024</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="I45" s="1" t="s">
         <v>95</v>
@@ -1728,9 +1713,6 @@
       <c r="F47" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="G47" s="1" t="s">
-        <v>106</v>
-      </c>
       <c r="I47" s="1" t="s">
         <v>96</v>
       </c>
@@ -1746,16 +1728,13 @@
         <v>2024</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F48" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="G48" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="I48" s="1" t="s">
         <v>95</v>
@@ -1780,9 +1759,6 @@
       <c r="F49" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="G49" s="1" t="s">
-        <v>107</v>
-      </c>
       <c r="I49" s="1" t="s">
         <v>96</v>
       </c>
@@ -1804,10 +1780,7 @@
         <v>73</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="G50" s="1" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="I50" s="1" t="s">
         <v>99</v>
@@ -1832,9 +1805,6 @@
       <c r="F51" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="G51" s="1" t="s">
-        <v>112</v>
-      </c>
       <c r="I51" s="1" t="s">
         <v>96</v>
       </c>
@@ -1887,7 +1857,7 @@
     </row>
     <row r="54" spans="1:9" ht="136" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B54" s="1">
         <v>2026</v>
@@ -1896,21 +1866,21 @@
         <v>2026</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B55" s="1">
         <v>2025</v>
@@ -1919,21 +1889,21 @@
         <v>2025</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="56" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B56" s="1">
         <v>2025</v>
@@ -1942,21 +1912,21 @@
         <v>2025</v>
       </c>
       <c r="D56" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E56" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="G56" s="1" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B57" s="1">
         <v>2025</v>
@@ -1965,21 +1935,21 @@
         <v>2025</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
     </row>
     <row r="58" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B58" s="1">
         <v>2025</v>
@@ -1988,21 +1958,21 @@
         <v>2025</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="59" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B59" s="1">
         <v>2025</v>
@@ -2011,21 +1981,21 @@
         <v>2025</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="60" spans="1:9" ht="85" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B60" s="1">
         <v>2024</v>
@@ -2034,21 +2004,21 @@
         <v>2024</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="61" spans="1:9" ht="136" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B61" s="1">
         <v>2024</v>
@@ -2057,16 +2027,16 @@
         <v>2024</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ASQ Kern dashboard update
</commit_message>
<xml_diff>
--- a/data/cv_entries.xlsx
+++ b/data/cv_entries.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimwright/Desktop/Resume/wright_cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B58EA9AD-27DA-E848-B503-047BC173AFD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D88B02-AEEE-6D4F-87D2-A5E9D3DDC7C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16160" xr2:uid="{C4D43CE4-6AA2-144D-A346-CE8B2E756935}"/>
   </bookViews>
@@ -423,16 +423,7 @@
     <t>https://jim-asr.shinyapps.io/yuba_priorities_map/</t>
   </si>
   <si>
-    <t>First 5 Kern ASQ Results, FY 2024-25</t>
-  </si>
-  <si>
     <t>Developed dashboard for First 5 Siskiyou to analyze geographic trends in results to Dolly Parton Imagination Library participant survey.</t>
-  </si>
-  <si>
-    <t>Developed dashboard to display countywide results from Ages and Stages Questionnaire administered during 2024-25 fiscal year.</t>
-  </si>
-  <si>
-    <t>https://jim-asr.shinyapps.io/F5Kern_ASQResults_FY24-25_dashboard/</t>
   </si>
   <si>
     <t>First 5 Kern Immunization Coalition Parent Survey</t>
@@ -479,6 +470,15 @@
   </si>
   <si>
     <t>https://jim-asr.shinyapps.io/F5Siskiyou_ELA_Readiness_Dashboard/</t>
+  </si>
+  <si>
+    <t>First 5 Kern ASQ Results, FY 2024-25 and 2025-26</t>
+  </si>
+  <si>
+    <t>https://jim-asr.shinyapps.io/F5Kern_ASQResults/</t>
+  </si>
+  <si>
+    <t>Developed dashboard to display countywide results from Ages and Stages Questionnaire administered during 2024-25 and 2025-26 fiscal years.</t>
   </si>
 </sst>
 </file>
@@ -957,13 +957,13 @@
         <v>15</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="409.5" x14ac:dyDescent="0.2">
@@ -1636,13 +1636,13 @@
         <v>15</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="I44" s="1" t="s">
         <v>115</v>
@@ -1866,16 +1866,16 @@
         <v>2026</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="119" x14ac:dyDescent="0.2">
@@ -1918,7 +1918,7 @@
         <v>111</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G56" s="1" t="s">
         <v>126</v>
@@ -1941,13 +1941,13 @@
         <v>111</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>121</v>
       </c>
@@ -1958,16 +1958,16 @@
         <v>2025</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
     </row>
     <row r="59" spans="1:9" ht="102" x14ac:dyDescent="0.2">
@@ -1981,13 +1981,13 @@
         <v>2025</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G59" s="1" t="s">
         <v>120</v>
@@ -2004,13 +2004,13 @@
         <v>2024</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G60" s="3" t="s">
         <v>119</v>
@@ -2027,16 +2027,16 @@
         <v>2024</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
additional data viz added
</commit_message>
<xml_diff>
--- a/data/cv_entries.xlsx
+++ b/data/cv_entries.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimwright/Desktop/Resume/wright_cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D88B02-AEEE-6D4F-87D2-A5E9D3DDC7C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF1545E-5802-7643-B07D-E64918F6518D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16160" xr2:uid="{C4D43CE4-6AA2-144D-A346-CE8B2E756935}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16180" xr2:uid="{C4D43CE4-6AA2-144D-A346-CE8B2E756935}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="154">
   <si>
     <t>type</t>
   </si>
@@ -479,6 +479,24 @@
   </si>
   <si>
     <t>Developed dashboard to display countywide results from Ages and Stages Questionnaire administered during 2024-25 and 2025-26 fiscal years.</t>
+  </si>
+  <si>
+    <t>Community Pathway Landscape Analysis</t>
+  </si>
+  <si>
+    <t>Developed a dashboard to support comparison of Sacramento County Community Pathways priority ZIP codes to countywide indicators from the COM map exports.</t>
+  </si>
+  <si>
+    <t>Yakama Nation Housing Needs Survey</t>
+  </si>
+  <si>
+    <t>Developed dashboard to display results from the Yakama Nation Housing Needs Survey.</t>
+  </si>
+  <si>
+    <t>https://jim-asr.shinyapps.io/CommPathLandscape/</t>
+  </si>
+  <si>
+    <t>https://jim-asr.shinyapps.io/YNHA_Survey_Analysis/</t>
   </si>
 </sst>
 </file>
@@ -849,7 +867,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8559F42B-99AA-F44B-B1DC-6C413C767572}">
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="16384" width="20.83203125" style="1"/>
@@ -1855,7 +1873,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="136" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:9" ht="68" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>121</v>
       </c>
@@ -1866,65 +1884,65 @@
         <v>2026</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="136" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>121</v>
       </c>
       <c r="B55" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C55" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>122</v>
+        <v>148</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>123</v>
+        <v>149</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="136" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>121</v>
       </c>
       <c r="B56" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C56" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>125</v>
+        <v>142</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>121</v>
       </c>
@@ -1935,16 +1953,16 @@
         <v>2025</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="58" spans="1:9" ht="119" x14ac:dyDescent="0.2">
@@ -1958,16 +1976,16 @@
         <v>2025</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>146</v>
+        <v>126</v>
       </c>
     </row>
     <row r="59" spans="1:9" ht="102" x14ac:dyDescent="0.2">
@@ -1981,61 +1999,107 @@
         <v>2025</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" ht="85" x14ac:dyDescent="0.2">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>121</v>
       </c>
       <c r="B60" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C60" s="1">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="G60" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" ht="136" x14ac:dyDescent="0.2">
+        <v>147</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>121</v>
       </c>
       <c r="B61" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C61" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F61" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" ht="85" x14ac:dyDescent="0.2">
+      <c r="A62" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B62" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C62" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="G62" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" ht="136" x14ac:dyDescent="0.2">
+      <c r="A63" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B63" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C63" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F63" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="G61" s="1" t="s">
+      <c r="G63" s="1" t="s">
         <v>135</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Siskiyou DPIL map update
</commit_message>
<xml_diff>
--- a/data/cv_entries.xlsx
+++ b/data/cv_entries.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimwright/Desktop/Resume/wright_cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF1545E-5802-7643-B07D-E64918F6518D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6077E8A0-2724-444E-9637-A167A169FD22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16180" xr2:uid="{C4D43CE4-6AA2-144D-A346-CE8B2E756935}"/>
   </bookViews>
@@ -414,9 +414,6 @@
     <t>First 5 Siskiyou Dolly Parton Imagination Library Survey</t>
   </si>
   <si>
-    <t>https://jim-asr.shinyapps.io/F5Siskiyou_DPIL_FY2025-26/</t>
-  </si>
-  <si>
     <t>First 5 Yuba Strategic Planning Community Survey</t>
   </si>
   <si>
@@ -497,6 +494,9 @@
   </si>
   <si>
     <t>https://jim-asr.shinyapps.io/YNHA_Survey_Analysis/</t>
+  </si>
+  <si>
+    <t>https://jim-asr.shinyapps.io/F5Siskiyou_DPIL_SurveyResults/</t>
   </si>
 </sst>
 </file>
@@ -975,13 +975,13 @@
         <v>15</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="409.5" x14ac:dyDescent="0.2">
@@ -1654,13 +1654,13 @@
         <v>15</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I44" s="1" t="s">
         <v>115</v>
@@ -1884,16 +1884,16 @@
         <v>2026</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="136" x14ac:dyDescent="0.2">
@@ -1907,16 +1907,16 @@
         <v>2026</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="56" spans="1:9" ht="136" x14ac:dyDescent="0.2">
@@ -1930,16 +1930,16 @@
         <v>2026</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F56" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="G56" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="119" x14ac:dyDescent="0.2">
@@ -1973,7 +1973,7 @@
         <v>2025</v>
       </c>
       <c r="C58" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D58" s="1" t="s">
         <v>125</v>
@@ -1982,10 +1982,10 @@
         <v>111</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="59" spans="1:9" ht="102" x14ac:dyDescent="0.2">
@@ -1999,16 +1999,16 @@
         <v>2025</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="60" spans="1:9" ht="119" x14ac:dyDescent="0.2">
@@ -2022,16 +2022,16 @@
         <v>2026</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="61" spans="1:9" ht="102" x14ac:dyDescent="0.2">
@@ -2045,13 +2045,13 @@
         <v>2025</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G61" s="1" t="s">
         <v>120</v>
@@ -2068,13 +2068,13 @@
         <v>2024</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G62" s="3" t="s">
         <v>119</v>
@@ -2091,16 +2091,16 @@
         <v>2024</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F63" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="G63" s="1" t="s">
         <v>134</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -2110,6 +2110,7 @@
     <hyperlink ref="G20" r:id="rId3" xr:uid="{A592B2D5-64F7-D24F-B190-D84D29F1718E}"/>
     <hyperlink ref="D20" r:id="rId4" xr:uid="{D42F41A6-5D73-B344-9F8A-BD6292306C55}"/>
     <hyperlink ref="F17" r:id="rId5" xr:uid="{9FC96BBB-E6A2-B445-A8BC-D5C33750B0BD}"/>
+    <hyperlink ref="G58" r:id="rId6" xr:uid="{BB18FF59-8C70-DC42-BE0F-0500E7BCE0F7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
additional data viz - first 5 kern
</commit_message>
<xml_diff>
--- a/data/cv_entries.xlsx
+++ b/data/cv_entries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimwright/Desktop/Resume/wright_cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03A518F6-F467-4247-88D8-14BDF7E9AE77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C29F22EA-420D-9840-B848-FE295E73FCE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16180" xr2:uid="{C4D43CE4-6AA2-144D-A346-CE8B2E756935}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="160">
   <si>
     <t>type</t>
   </si>
@@ -506,6 +506,15 @@
   </si>
   <si>
     <t>https://jim-asr.shinyapps.io/sccfc_pantrysoft/</t>
+  </si>
+  <si>
+    <t>First 5 Kern Fatherhood Survey</t>
+  </si>
+  <si>
+    <t>Developed dashboard to display results from First 5 Kern Fatherhood Survey.</t>
+  </si>
+  <si>
+    <t>https://jim-asr.shinyapps.io/KernFatherhoodSurvey/</t>
   </si>
 </sst>
 </file>
@@ -876,7 +885,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8559F42B-99AA-F44B-B1DC-6C413C767572}">
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="16384" width="20.83203125" style="1"/>
@@ -1893,19 +1902,19 @@
         <v>2026</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="68" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>121</v>
       </c>
@@ -1916,19 +1925,19 @@
         <v>2026</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>125</v>
+        <v>154</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+        <v>155</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>121</v>
       </c>
@@ -1939,19 +1948,19 @@
         <v>2026</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>149</v>
+        <v>125</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" ht="136" x14ac:dyDescent="0.2">
+        <v>128</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="68" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>121</v>
       </c>
@@ -1962,16 +1971,16 @@
         <v>2026</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="58" spans="1:9" ht="136" x14ac:dyDescent="0.2">
@@ -1985,42 +1994,42 @@
         <v>2026</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="136" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>121</v>
       </c>
       <c r="B59" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C59" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>121</v>
       </c>
@@ -2031,19 +2040,19 @@
         <v>2025</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>121</v>
       </c>
@@ -2051,22 +2060,22 @@
         <v>2025</v>
       </c>
       <c r="C61" s="1">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>144</v>
+        <v>126</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>121</v>
       </c>
@@ -2074,45 +2083,45 @@
         <v>2025</v>
       </c>
       <c r="C62" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" ht="85" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>121</v>
       </c>
       <c r="B63" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C63" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="G63" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" ht="136" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" ht="85" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>121</v>
       </c>
@@ -2123,15 +2132,38 @@
         <v>2024</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F64" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="G64" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="136" x14ac:dyDescent="0.2">
+      <c r="A65" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B65" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C65" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F65" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G64" s="1" t="s">
+      <c r="G65" s="1" t="s">
         <v>134</v>
       </c>
     </row>
@@ -2142,7 +2174,7 @@
     <hyperlink ref="G20" r:id="rId3" xr:uid="{A592B2D5-64F7-D24F-B190-D84D29F1718E}"/>
     <hyperlink ref="D20" r:id="rId4" xr:uid="{D42F41A6-5D73-B344-9F8A-BD6292306C55}"/>
     <hyperlink ref="F17" r:id="rId5" xr:uid="{9FC96BBB-E6A2-B445-A8BC-D5C33750B0BD}"/>
-    <hyperlink ref="G55" r:id="rId6" xr:uid="{28F1EDDD-1C35-AC45-B7F9-6B83091A5EF4}"/>
+    <hyperlink ref="G56" r:id="rId6" xr:uid="{28F1EDDD-1C35-AC45-B7F9-6B83091A5EF4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>